<commit_message>
chore: update TID sample template with settlement config columns
</commit_message>
<xml_diff>
--- a/src/main/resources/sample/tids_sample.xlsx
+++ b/src/main/resources/sample/tids_sample.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,8 +49,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,68 +417,142 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:V2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="20" customWidth="1" min="20" max="20"/>
+    <col width="20" customWidth="1" min="21" max="21"/>
+    <col width="20" customWidth="1" min="22" max="22"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>terminalId</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>merchantId</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>merchantName</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>bankCode</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>bankAccNo</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>merchantCategoryCode</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>stateCode</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>merchantPhysicalAddr</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>merchantAddressLgaCode</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>processor</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>settlementType</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>settlementTime</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>settlementDays</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>settlementAccountName</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>settlementBankName</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>settlementAccountNumber</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>settlementAccountType</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>mscPosPercentage</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>instantTransferFee</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>monthlyTerminalFee</t>
         </is>
       </c>
     </row>
@@ -496,7 +574,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>IKECHI.IKWUONYE@IRPAY.NG</t>
+          <t>merchant@example.com</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -526,7 +604,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>3A OLARENWAJU NINALOWO ST LEKKI 1</t>
+          <t>3A OLARENWAJU ST LEKKI</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -535,6 +613,56 @@
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>T+1</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>5:00 PM Daily</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Monday - Friday</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>IRCMS LIMITED</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Access Bank</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>1305063834</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Current Account</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>0.50</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>50.00</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>1000.00</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>